<commit_message>
cambios en los resúmenes
</commit_message>
<xml_diff>
--- a/ignore/alma_bat.xlsx
+++ b/ignore/alma_bat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanj\Documents\GitHub\alma\ignore\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8DB192-64AD-434C-A4E0-4B1FC9C43B36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E55CB8A-2E8E-4020-B392-F0B336E3B316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="75">
   <si>
     <t>A dónde lo huido</t>
   </si>
@@ -734,7 +734,12 @@
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">

</xml_diff>